<commit_message>
Agenda recorrente, calendario dashboard e recebimento de mensalidades
</commit_message>
<xml_diff>
--- a/relatorio_mensalidades.xlsx
+++ b/relatorio_mensalidades.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,25 +446,325 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>05/2026</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>320</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-05-25</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Pago</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>06/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>320</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>07/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>320</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-07-25</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>08/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>320</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>09/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>320</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>320</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-10-25</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>11/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>320</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-11-25</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>12/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>320</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-12-25</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>01/2027</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>320</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2027-01-25</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>02/2027</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>320</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2027-02-25</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>03/2027</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>320</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2027-03-25</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Aline Canfield Martins</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>04/2027</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>320</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2027-04-25</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>Michel Garcia de Sousa</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Junho/2026</t>
         </is>
       </c>
-      <c r="C2" t="n">
+      <c r="C14" t="n">
         <v>100</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>2026-06-15</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Pago</t>
         </is>
       </c>
     </row>

</xml_diff>